<commit_message>
wip(aset): keputusan pemilik untuk monitoring (tanpa unit, izin baca, beda lokasi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/laporan-monitoring-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/laporan-monitoring-aset/standar.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Monitoring aset" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitoring aset'!$A$11:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitoring aset'!$A$11:$R$11</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="66">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>${baris.kondisi_sistem}</t>
+  </si>
+  <si>
+    <t>Lokasi tercatat</t>
+  </si>
+  <si>
+    <t>${baris.lokasi_tercatat}</t>
   </si>
   <si>
     <t>Keberadaan fisik</t>
@@ -634,7 +640,7 @@
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -645,18 +651,19 @@
     <col min="6" max="6" width="28" customWidth="true" style="0"/>
     <col min="7" max="7" width="26" customWidth="true" style="0"/>
     <col min="8" max="8" width="16" customWidth="true" style="0"/>
-    <col min="9" max="9" width="14" customWidth="true" style="0"/>
-    <col min="10" max="10" width="16" customWidth="true" style="0"/>
+    <col min="9" max="9" width="22" customWidth="true" style="0"/>
+    <col min="10" max="10" width="14" customWidth="true" style="0"/>
     <col min="11" max="11" width="16" customWidth="true" style="0"/>
-    <col min="12" max="12" width="30" customWidth="true" style="0"/>
-    <col min="13" max="13" width="18" customWidth="true" style="0"/>
+    <col min="12" max="12" width="16" customWidth="true" style="0"/>
+    <col min="13" max="13" width="30" customWidth="true" style="0"/>
     <col min="14" max="14" width="18" customWidth="true" style="0"/>
     <col min="15" max="15" width="18" customWidth="true" style="0"/>
-    <col min="16" max="16" width="22" customWidth="true" style="0"/>
+    <col min="16" max="16" width="18" customWidth="true" style="0"/>
     <col min="17" max="17" width="22" customWidth="true" style="0"/>
+    <col min="18" max="18" width="22" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" customHeight="1" ht="22">
+    <row r="1" spans="1:18" customHeight="1" ht="22">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -677,11 +684,12 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1"/>
+      <c r="R1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:17" customHeight="1" ht="24">
+    <row r="2" spans="1:18" customHeight="1" ht="24">
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
@@ -699,8 +707,9 @@
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
-    </row>
-    <row r="3" spans="1:17" customHeight="1" ht="22">
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="1:18" customHeight="1" ht="22">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
         <v>3</v>
@@ -719,14 +728,15 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
-      <c r="Q3" s="3"/>
-    </row>
-    <row r="5" spans="1:17">
+      <c r="Q3" s="4"/>
+      <c r="R3" s="3"/>
+    </row>
+    <row r="5" spans="1:18">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:18">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -746,7 +756,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:18">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -766,7 +776,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:18">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -786,7 +796,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:18">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -806,7 +816,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:17" customHeight="1" ht="32">
+    <row r="11" spans="1:18" customHeight="1" ht="32">
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
@@ -835,10 +845,10 @@
         <v>46</v>
       </c>
       <c r="J11" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K11" s="7" t="s">
         <v>20</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>49</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>51</v>
@@ -853,13 +863,16 @@
         <v>57</v>
       </c>
       <c r="P11" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="Q11" s="7" t="s">
+      <c r="R11" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:18">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -888,7 +901,7 @@
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K12" t="s">
         <v>50</v>
@@ -906,15 +919,18 @@
         <v>58</v>
       </c>
       <c r="P12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q12" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17">
+        <v>61</v>
+      </c>
+      <c r="R12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18">
       <c r="A13" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -927,25 +943,26 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
       <c r="L13" s="8"/>
-      <c r="M13" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="P13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8" t="s">
+        <v>65</v>
+      </c>
       <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A11:Q11"/>
+  <autoFilter ref="A11:R11"/>
   <mergeCells>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:P1"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="B3:P3"/>
-    <mergeCell ref="Q1:Q3"/>
-    <mergeCell ref="A13:L13"/>
+    <mergeCell ref="B1:Q1"/>
+    <mergeCell ref="B2:Q2"/>
+    <mergeCell ref="B3:Q3"/>
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="A13:M13"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>